<commit_message>
Split player popup into Sponsors and Money Collected
Sponsor payments now show once, under the sponsor, instead of again in a
payments list. Everything else (family, deposit, table collections) is
under Money Collected. Each section shows a subtotal, and they add up to
the player's total. Adds a split table-collection example and instructions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/Storm-Branson-Tracker.xlsx
+++ b/template/Storm-Branson-Tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -517,63 +517,77 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Use Sponsor for company donations, Family for money from the player's family, Fundraiser for event money.</t>
+          <t xml:space="preserve">        Use Sponsor for money from a company (it shows under the player's Sponsors), Family for family money, Fundraiser for table/event money.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Table collections (e.g. two boys at a Dunkin' Donuts table): split the money and add ONE ROW PER BOY with his share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Put the same "From" on each (e.g. Dunkin' Donuts table) and a note like "Split with Jake ($125 total)".</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  Every payment, including the deposit, counts toward the player's $1,000 bucket.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>SPONSORS tab: the companies each player is asking for donations.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  Status: Asked, Pledged, Paid, or Declined. Pledged Amount: what they promised (optional).</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  When the money actually arrives, ALSO add it on the Payments tab, with the same company name in "From".</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>PLAYERS tab: the roster. Add or remove rows and the dashboard follows. Keep names spelled exactly the same everywhere.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>SETTINGS tab: goal per player, deposit amount, deposit deadline (type it like 3/1/2027), team discount.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Don't rename the tabs or the column headers in row 1. The dashboard finds data by those names.</t>
         </is>

</xml_diff>